<commit_message>
.gitignore file added for ignored version control on few folders Firmware, Logs, ScreenShots, & Reports
And Readme.txt information added

Signed-off-by: sathishs28 <sathishgesh28@gmail.com>
</commit_message>
<xml_diff>
--- a/TestData/Data_Driven_Test.xlsx
+++ b/TestData/Data_Driven_Test.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="WAN" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="122211"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
   <si>
     <t>Username</t>
   </si>
@@ -64,6 +64,39 @@
   </si>
   <si>
     <t>adminad</t>
+  </si>
+  <si>
+    <t>VLAN ID</t>
+  </si>
+  <si>
+    <t>CHANNEL MODE</t>
+  </si>
+  <si>
+    <t>CONNECTION TYPE</t>
+  </si>
+  <si>
+    <t>Bridged</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Add New Bridge WAN</t>
+  </si>
+  <si>
+    <t>Add New IPoE WAN</t>
+  </si>
+  <si>
+    <t>IPoE</t>
+  </si>
+  <si>
+    <t>INTERNET_TR069</t>
+  </si>
+  <si>
+    <t>Add New PPPoE WAN</t>
+  </si>
+  <si>
+    <t>PPPoE</t>
   </si>
 </sst>
 </file>
@@ -105,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -115,6 +148,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -521,10 +557,101 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="4"/>
+    <col min="4" max="4" width="19.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1000</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="2">
+        <v>50</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2">
+        <v>200</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D4">
+      <formula1>"Bridged,IPoE,PPPoE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E4">
+      <formula1>"Other,TR069,INTERNET,INTERNET_TR069,VOICE,VOICE_TR069,VOICE_INTERNET,VOICE_INTERNET_TR069"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Test Data (Data_Driven_Test.xlsx) file updated WAN details and protected the sheet. Refer Readme.txt
And Test_003_New_WAN.py & Test_005_Add_PPPoE_WAN.py modified for getting WAN details from Data_Driven_Test.xlsx (Test Data). In feature tester can modify the WAN details.

And Readme.txt info added
</commit_message>
<xml_diff>
--- a/TestData/Data_Driven_Test.xlsx
+++ b/TestData/Data_Driven_Test.xlsx
@@ -11,12 +11,12 @@
     <sheet name="WAN" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
   <si>
     <t>Username</t>
   </si>
@@ -30,21 +30,12 @@
     <t>admin</t>
   </si>
   <si>
-    <t>system</t>
-  </si>
-  <si>
     <t>PASS</t>
   </si>
   <si>
-    <t>adminsd</t>
-  </si>
-  <si>
     <t>FAIL</t>
   </si>
   <si>
-    <t>system12</t>
-  </si>
-  <si>
     <t>Test Case</t>
   </si>
   <si>
@@ -63,9 +54,6 @@
     <t>S.NO</t>
   </si>
   <si>
-    <t>adminad</t>
-  </si>
-  <si>
     <t>VLAN ID</t>
   </si>
   <si>
@@ -97,16 +85,62 @@
   </si>
   <si>
     <t>PPPoE</t>
+  </si>
+  <si>
+    <t>Ovt@12345</t>
+  </si>
+  <si>
+    <t>adminaddf</t>
+  </si>
+  <si>
+    <t>system12fgf</t>
+  </si>
+  <si>
+    <t>system12dgf</t>
+  </si>
+  <si>
+    <t>adminsdsfgd</t>
+  </si>
+  <si>
+    <t>PPP USERNAME</t>
+  </si>
+  <si>
+    <t>PPP PASSWORD</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>automation@vlan200</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>Note: Edit/Change the valid username &amp; password only, remainings you can't editable
+Allowed Cells - C2 &amp; D2</t>
+  </si>
+  <si>
+    <t>Note: Edit/Change the WAN configuration details, remainings you can't editable
+Allowed columns - C, E, F, &amp; G</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -135,10 +169,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -152,8 +187,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -453,24 +501,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
     <col min="2" max="2" width="32.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.140625" style="2"/>
     <col min="6" max="6" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -482,166 +530,238 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>3</v>
+        <v>9</v>
+      </c>
+      <c r="C3" s="3" t="str">
+        <f>C2</f>
+        <v>admin</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>4</v>
+        <v>24</v>
+      </c>
+      <c r="D4" s="3" t="str">
+        <f>D2</f>
+        <v>Ovt@12345</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>7</v>
-      </c>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
     </row>
   </sheetData>
+  <sheetProtection password="8584" sheet="1" objects="1" scenarios="1"/>
+  <protectedRanges>
+    <protectedRange password="CCEE" sqref="C2:D2" name="Range1" securityDescriptor="O:WDG:WDD:(A;;CC;;;LA)"/>
+  </protectedRanges>
+  <mergeCells count="1">
+    <mergeCell ref="A8:I8"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="32.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.140625" style="4"/>
     <col min="4" max="4" width="19.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C2" s="2">
         <v>1000</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C3" s="2">
         <v>50</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C4" s="2">
         <v>200</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
     </row>
+    <row r="7" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+    </row>
   </sheetData>
+  <sheetProtection password="8584" sheet="1" objects="1" scenarios="1"/>
+  <protectedRanges>
+    <protectedRange password="CCEE" sqref="C2:C4 E2:E4 F4:G4" name="Range1" securityDescriptor="O:WDG:WDD:(A;;CC;;;LA)"/>
+  </protectedRanges>
+  <mergeCells count="1">
+    <mergeCell ref="A7:I7"/>
+  </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D4">
       <formula1>"Bridged,IPoE,PPPoE"</formula1>
@@ -650,8 +770,11 @@
       <formula1>"Other,TR069,INTERNET,INTERNET_TR069,VOICE,VOICE_TR069,VOICE_INTERNET,VOICE_INTERNET_TR069"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="F4" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>